<commit_message>
edits to column names in template, minor text changes
</commit_message>
<xml_diff>
--- a/templates/blank_context_template_sep2026.xlsx
+++ b/templates/blank_context_template_sep2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10914"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FE0325-21FF-B540-AFF3-C9DED06E2A88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36DB2A15-C5BB-354B-846A-2C0480E630A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2760" yWindow="1580" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2480" yWindow="940" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Guide" sheetId="8" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="595" uniqueCount="499">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="602" uniqueCount="499">
   <si>
     <t>lith_comp</t>
   </si>
@@ -647,19 +647,10 @@
     <t>interpreted age justification*</t>
   </si>
   <si>
-    <t>section_name*</t>
-  </si>
-  <si>
-    <t>site_type*</t>
-  </si>
-  <si>
     <t>latitude*</t>
   </si>
   <si>
     <t>longitude*</t>
-  </si>
-  <si>
-    <t>metamorphic_bin*</t>
   </si>
   <si>
     <r>
@@ -1249,26 +1240,6 @@
     <t>mineral (phosphate)</t>
   </si>
   <si>
-    <t xml:space="preserve">Environments are divided into three bins - inner shelf/outer shelf/basinal  - according to the following criteria (1-3 from Sperling et al. 2015), plus Lacustrine, Fluvial, and Estuarine. 
-1) Environment 1/Inner Shelf: Sample interbedded with abundant shallow-water
-indicators. This includes clastic beds with wave-generated sedimentary
-structures as well as shallow-water carbonates such as stromatolites, oolites,
-and rip-up conglomerates. Evidence of exposure—i.e. mudcracks, karsting,
-teepee structures—are often in relatively close stratigraphic proximity on the
-meters to 10s of meters scale.
-2) Environment 2/Outer Shelf: Sample from sequences that generally show little
-wave activity, but with occasional evidence for storm and/or wave activity,
-such as hummocky cross-stratified sands encased in shales. Evidence for
-exposure is not in close stratigraphic proximity.
-3) Environment 3/Basinal: Sample from successions with no evidence for any storm
-and/or wave activity for an appreciable (i.e. &gt;50 m) stratigraphic distance.
-Generally located considerably basin-ward of shallower-water facies.
-4) Lacustrine
-5) Fluvial
-6) Estuarine
-</t>
-  </si>
-  <si>
     <t xml:space="preserve">A more detailed category of depositional environment (added 2021). List of terms is from Macrostrat. These are listed as carbonate marine depositional environments, siliciclastic marine depositional environments, followed by fluvial, lacustrine, glacial, and other depositional environments.
 </t>
   </si>
@@ -1751,6 +1722,35 @@
   </si>
   <si>
     <t>Any significant details that were not captured in the preceding columns. For example, alternative site names, details relating to how the lat-long was gathered.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environments are divided into three bins - inner shelf/outer shelf/basinal  - according to the following criteria (1-3 from Sperling et al. 2015), plus Lacustrine, Fluvial, and Estuarine. 
+1) Inner Shelf: Sample interbedded with abundant shallow-water
+indicators. This includes clastic beds with wave-generated sedimentary
+structures as well as shallow-water carbonates such as stromatolites, oolites,
+and rip-up conglomerates. Evidence of exposure—i.e. mudcracks, karsting,
+teepee structures—are often in relatively close stratigraphic proximity on the
+meters to 10s of meters scale.
+2) Outer Shelf: Sample from sequences that generally show little
+wave activity, but with occasional evidence for storm and/or wave activity,
+such as hummocky cross-stratified sands encased in shales. Evidence for
+exposure is not in close stratigraphic proximity.
+3) Basinal: Sample from successions with no evidence for any storm
+and/or wave activity for an appreciable (i.e. &gt;50 m) stratigraphic distance.
+Generally located considerably basin-ward of shallower-water facies.
+4) Lacustrine
+5) Fluvial
+6) Estuarine
+</t>
+  </si>
+  <si>
+    <t>site type*</t>
+  </si>
+  <si>
+    <t>craton or terrane</t>
+  </si>
+  <si>
+    <t>metamorphic bin*</t>
   </si>
 </sst>
 </file>
@@ -2214,14 +2214,15 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2232,7 +2233,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="201">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -2437,47 +2437,7 @@
     <cellStyle name="Hyperlink" xfId="199" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2843,19 +2803,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="83" customHeight="1">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="49" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
       <c r="D1" s="45"/>
     </row>
     <row r="2" spans="1:4" s="8" customFormat="1" ht="148" customHeight="1">
-      <c r="A2" s="46" t="s">
-        <v>202</v>
-      </c>
-      <c r="B2" s="46"/>
-      <c r="C2" s="46"/>
+      <c r="A2" s="48" t="s">
+        <v>199</v>
+      </c>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
       <c r="D2" s="26"/>
     </row>
     <row r="5" spans="1:4" ht="19">
@@ -2905,10 +2865,10 @@
     </row>
     <row r="11" spans="1:4" ht="34">
       <c r="A11" s="7" t="s">
-        <v>458</v>
+        <v>454</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="170">
@@ -2924,7 +2884,7 @@
         <v>106</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>477</v>
+        <v>473</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="51">
@@ -2932,7 +2892,7 @@
         <v>138</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>476</v>
+        <v>472</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -2940,7 +2900,7 @@
         <v>115</v>
       </c>
       <c r="B15" t="s">
-        <v>478</v>
+        <v>474</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="19">
@@ -2953,15 +2913,15 @@
         <v>124</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>479</v>
+        <v>475</v>
       </c>
     </row>
     <row r="20" spans="1:4" ht="170">
       <c r="A20" s="15" t="s">
-        <v>459</v>
+        <v>455</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>480</v>
+        <v>476</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="409.6">
@@ -2969,16 +2929,16 @@
         <v>161</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>363</v>
+        <v>495</v>
       </c>
       <c r="C21" s="7"/>
     </row>
     <row r="22" spans="1:4" ht="68">
       <c r="A22" s="15" t="s">
-        <v>460</v>
+        <v>456</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="C22" s="7"/>
     </row>
@@ -2995,7 +2955,7 @@
         <v>136</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
     </row>
     <row r="25" spans="1:4">
@@ -3036,7 +2996,7 @@
         <v>130</v>
       </c>
       <c r="B29" s="16" t="s">
-        <v>461</v>
+        <v>457</v>
       </c>
     </row>
     <row r="30" spans="1:4" ht="51">
@@ -3044,7 +3004,7 @@
         <v>3</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="51">
@@ -3052,7 +3012,7 @@
         <v>133</v>
       </c>
       <c r="B31" s="16" t="s">
-        <v>481</v>
+        <v>477</v>
       </c>
       <c r="D31" s="2"/>
     </row>
@@ -3061,7 +3021,7 @@
         <v>163</v>
       </c>
       <c r="B32" s="16" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="51">
@@ -3074,23 +3034,23 @@
     </row>
     <row r="35" spans="1:2" ht="19">
       <c r="A35" s="9" t="s">
-        <v>366</v>
+        <v>362</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="102">
       <c r="A36" s="15" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>465</v>
+        <v>461</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="51">
       <c r="A37" s="15" t="s">
-        <v>463</v>
+        <v>459</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>482</v>
+        <v>478</v>
       </c>
     </row>
   </sheetData>
@@ -3133,10 +3093,10 @@
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="38" customHeight="1">
       <c r="A1" s="12" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>198</v>
+        <v>496</v>
       </c>
       <c r="C1" s="17" t="s">
         <v>111</v>
@@ -3151,10 +3111,10 @@
         <v>114</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="I1" s="17" t="s">
         <v>139</v>
@@ -3163,7 +3123,7 @@
         <v>123</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>105</v>
+        <v>497</v>
       </c>
       <c r="L1" s="13" t="s">
         <v>117</v>
@@ -3172,7 +3132,7 @@
         <v>116</v>
       </c>
       <c r="N1" s="18" t="s">
-        <v>201</v>
+        <v>498</v>
       </c>
       <c r="O1" s="20" t="s">
         <v>131</v>
@@ -3184,7 +3144,7 @@
         <v>106</v>
       </c>
       <c r="R1" s="20" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>115</v>
@@ -3213,7 +3173,7 @@
         <v>179</v>
       </c>
       <c r="J2" s="14" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>180</v>
@@ -3230,25 +3190,25 @@
       <c r="O2" s="21"/>
       <c r="P2" s="21"/>
       <c r="Q2" s="21" t="s">
-        <v>467</v>
+        <v>463</v>
       </c>
       <c r="R2" s="21" t="s">
-        <v>468</v>
+        <v>464</v>
       </c>
       <c r="S2" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="27" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="G3" s="35"/>
       <c r="H3" s="35"/>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="27" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="G4" s="35"/>
       <c r="H4" s="35"/>
@@ -3297,11 +3257,11 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:AA3"/>
+  <dimension ref="A1:AA12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" style="52" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" style="46" customWidth="1"/>
     <col min="3" max="3" width="38.33203125" customWidth="1"/>
     <col min="4" max="4" width="44" customWidth="1"/>
     <col min="5" max="5" width="29.5" customWidth="1"/>
@@ -3348,10 +3308,10 @@
       <c r="R1" s="43"/>
       <c r="S1" s="43"/>
       <c r="T1" s="43"/>
-      <c r="U1" s="48" t="s">
+      <c r="U1" s="47" t="s">
         <v>133</v>
       </c>
-      <c r="V1" s="48"/>
+      <c r="V1" s="47"/>
       <c r="W1" s="24"/>
       <c r="X1" s="24"/>
       <c r="Y1" s="25"/>
@@ -3359,7 +3319,7 @@
     </row>
     <row r="2" spans="1:27" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="A2" s="34" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="B2" s="28" t="s">
         <v>188</v>
@@ -3371,7 +3331,7 @@
         <v>190</v>
       </c>
       <c r="E2" s="29" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="F2" s="11" t="s">
         <v>191</v>
@@ -3380,7 +3340,7 @@
         <v>192</v>
       </c>
       <c r="H2" s="32" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="I2" s="11" t="s">
         <v>125</v>
@@ -3425,16 +3385,16 @@
         <v>196</v>
       </c>
       <c r="W2" s="13" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="X2" s="13" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="Y2" s="20" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="Z2" s="20" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="AA2" s="1" t="s">
         <v>115</v>
@@ -3442,16 +3402,16 @@
     </row>
     <row r="3" spans="1:27" ht="17">
       <c r="A3" s="21" t="s">
-        <v>474</v>
+        <v>470</v>
       </c>
       <c r="B3" s="40" t="s">
-        <v>473</v>
+        <v>469</v>
       </c>
       <c r="C3" s="41" t="s">
-        <v>372</v>
+        <v>368</v>
       </c>
       <c r="D3" s="40" t="s">
-        <v>495</v>
+        <v>491</v>
       </c>
       <c r="E3" s="33" t="s">
         <v>157</v>
@@ -3473,7 +3433,7 @@
         <v>159</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="M3" s="4" t="s">
         <v>157</v>
@@ -3489,34 +3449,69 @@
       </c>
       <c r="Q3" s="4"/>
       <c r="R3" s="4" t="s">
-        <v>367</v>
+        <v>363</v>
       </c>
       <c r="S3" s="4" t="s">
-        <v>373</v>
+        <v>369</v>
       </c>
       <c r="T3" s="4" t="s">
-        <v>374</v>
+        <v>370</v>
       </c>
       <c r="U3" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="Y3" s="21" t="s">
+        <v>467</v>
+      </c>
+      <c r="Z3" s="21" t="s">
         <v>466</v>
-      </c>
-      <c r="V3" s="5" t="s">
-        <v>469</v>
-      </c>
-      <c r="W3" s="5" t="s">
-        <v>466</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>466</v>
-      </c>
-      <c r="Y3" s="21" t="s">
-        <v>471</v>
-      </c>
-      <c r="Z3" s="21" t="s">
-        <v>470</v>
       </c>
       <c r="AA3" t="s">
         <v>183</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27">
+      <c r="O6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27">
+      <c r="O7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27">
+      <c r="O8" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27">
+      <c r="O9" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27">
+      <c r="O10" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27">
+      <c r="O11" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="12" spans="1:27">
+      <c r="O12" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -3612,10 +3607,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="37" t="s">
-        <v>462</v>
+        <v>458</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>464</v>
+        <v>460</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>115</v>
@@ -3623,13 +3618,13 @@
     </row>
     <row r="2" spans="1:3" s="16" customFormat="1" ht="35" customHeight="1">
       <c r="A2" s="38" t="s">
-        <v>472</v>
+        <v>468</v>
       </c>
       <c r="B2" s="39" t="s">
-        <v>475</v>
+        <v>471</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>457</v>
+        <v>453</v>
       </c>
     </row>
   </sheetData>
@@ -3665,7 +3660,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>392</v>
+        <v>388</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -3680,7 +3675,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -3735,7 +3730,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="17" spans="1:1">
@@ -3745,7 +3740,7 @@
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>396</v>
+        <v>392</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -3760,7 +3755,7 @@
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>390</v>
+        <v>386</v>
       </c>
     </row>
     <row r="22" spans="1:1">
@@ -3785,22 +3780,22 @@
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>385</v>
+        <v>381</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>381</v>
+        <v>377</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>384</v>
+        <v>380</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>376</v>
+        <v>372</v>
       </c>
     </row>
     <row r="30" spans="1:1">
@@ -3815,7 +3810,7 @@
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>382</v>
+        <v>378</v>
       </c>
     </row>
     <row r="33" spans="1:1">
@@ -3825,22 +3820,22 @@
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>391</v>
+        <v>387</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>379</v>
+        <v>375</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>378</v>
+        <v>374</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>389</v>
+        <v>385</v>
       </c>
     </row>
     <row r="38" spans="1:1">
@@ -3855,7 +3850,7 @@
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>398</v>
+        <v>394</v>
       </c>
     </row>
     <row r="41" spans="1:1">
@@ -3870,22 +3865,22 @@
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>380</v>
+        <v>376</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>387</v>
+        <v>383</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>383</v>
+        <v>379</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" t="s">
-        <v>375</v>
+        <v>371</v>
       </c>
     </row>
     <row r="47" spans="1:1">
@@ -3895,12 +3890,12 @@
     </row>
     <row r="48" spans="1:1">
       <c r="A48" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" t="s">
-        <v>393</v>
+        <v>389</v>
       </c>
     </row>
     <row r="50" spans="1:1">
@@ -3910,22 +3905,22 @@
     </row>
     <row r="51" spans="1:1">
       <c r="A51" t="s">
-        <v>377</v>
+        <v>373</v>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" t="s">
-        <v>395</v>
+        <v>391</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" t="s">
-        <v>400</v>
+        <v>396</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" t="s">
-        <v>397</v>
+        <v>393</v>
       </c>
     </row>
     <row r="55" spans="1:1">
@@ -3940,7 +3935,7 @@
     </row>
     <row r="57" spans="1:1">
       <c r="A57" t="s">
-        <v>399</v>
+        <v>395</v>
       </c>
     </row>
     <row r="58" spans="1:1">
@@ -3950,17 +3945,17 @@
     </row>
     <row r="59" spans="1:1">
       <c r="A59" t="s">
-        <v>394</v>
+        <v>390</v>
       </c>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" t="s">
-        <v>388</v>
+        <v>384</v>
       </c>
     </row>
     <row r="61" spans="1:1">
       <c r="A61" t="s">
-        <v>386</v>
+        <v>382</v>
       </c>
     </row>
   </sheetData>
@@ -3968,7 +3963,7 @@
     <sortCondition ref="A2:A61"/>
   </sortState>
   <conditionalFormatting sqref="A2:A61">
-    <cfRule type="duplicateValues" dxfId="5" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>
@@ -4006,49 +4001,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24">
-      <c r="A1" s="49" t="s">
-        <v>232</v>
-      </c>
-      <c r="B1" s="49"/>
-      <c r="C1" s="49"/>
-      <c r="D1" s="49"/>
+      <c r="A1" s="50" t="s">
+        <v>229</v>
+      </c>
+      <c r="B1" s="50"/>
+      <c r="C1" s="50"/>
+      <c r="D1" s="50"/>
       <c r="E1" s="14" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
-      <c r="H1" s="50" t="s">
-        <v>234</v>
-      </c>
-      <c r="I1" s="50"/>
-      <c r="J1" s="50"/>
+      <c r="H1" s="51" t="s">
+        <v>231</v>
+      </c>
+      <c r="I1" s="51"/>
+      <c r="J1" s="51"/>
       <c r="K1" s="5" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="L1" s="5"/>
       <c r="M1" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="N1" s="51" t="s">
-        <v>267</v>
-      </c>
-      <c r="O1" s="51"/>
-      <c r="P1" s="51"/>
-      <c r="Q1" s="51"/>
-      <c r="R1" s="51"/>
-      <c r="S1" s="49" t="s">
+      <c r="N1" s="52" t="s">
+        <v>264</v>
+      </c>
+      <c r="O1" s="52"/>
+      <c r="P1" s="52"/>
+      <c r="Q1" s="52"/>
+      <c r="R1" s="52"/>
+      <c r="S1" s="50" t="s">
         <v>142</v>
       </c>
-      <c r="T1" s="49"/>
-      <c r="U1" s="49"/>
+      <c r="T1" s="50"/>
+      <c r="U1" s="50"/>
       <c r="V1" s="19" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="W1" s="31" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>455</v>
+        <v>451</v>
       </c>
     </row>
     <row r="2" spans="1:24">
@@ -4098,7 +4093,7 @@
         <v>116</v>
       </c>
       <c r="X2" t="s">
-        <v>456</v>
+        <v>452</v>
       </c>
     </row>
     <row r="3" spans="1:24">
@@ -4136,7 +4131,7 @@
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="M3" t="s">
         <v>104</v>
@@ -4145,7 +4140,7 @@
         <v>1</v>
       </c>
       <c r="O3" s="23" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="S3">
         <v>1</v>
@@ -4157,13 +4152,13 @@
         <v>143</v>
       </c>
       <c r="V3" t="s">
-        <v>483</v>
+        <v>479</v>
       </c>
       <c r="W3" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="X3" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
     </row>
     <row r="4" spans="1:24">
@@ -4201,7 +4196,7 @@
         <v>2</v>
       </c>
       <c r="L4" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="M4" t="s">
         <v>110</v>
@@ -4222,13 +4217,13 @@
         <v>145</v>
       </c>
       <c r="V4" t="s">
-        <v>484</v>
+        <v>480</v>
       </c>
       <c r="W4" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="X4" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5" spans="1:24">
@@ -4266,16 +4261,16 @@
         <v>3</v>
       </c>
       <c r="L5" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="M5" t="s">
-        <v>494</v>
+        <v>490</v>
       </c>
       <c r="N5">
         <v>3</v>
       </c>
       <c r="O5" s="23" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="S5">
         <v>3</v>
@@ -4287,13 +4282,13 @@
         <v>147</v>
       </c>
       <c r="V5" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="W5" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="X5" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
     </row>
     <row r="6" spans="1:24">
@@ -4337,16 +4332,16 @@
         <v>4</v>
       </c>
       <c r="O6" s="23" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="V6" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="W6" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="X6" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="7" spans="1:24">
@@ -4384,13 +4379,13 @@
         <v>121</v>
       </c>
       <c r="V7" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="W7" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="X7" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
     </row>
     <row r="8" spans="1:24">
@@ -4410,7 +4405,7 @@
         <v>6</v>
       </c>
       <c r="I8" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="J8" t="s">
         <v>31</v>
@@ -4419,7 +4414,7 @@
         <v>6</v>
       </c>
       <c r="L8" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="N8">
         <v>6</v>
@@ -4428,13 +4423,13 @@
         <v>122</v>
       </c>
       <c r="V8" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="W8" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="X8" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="9" spans="1:24">
@@ -4463,13 +4458,13 @@
         <v>118</v>
       </c>
       <c r="V9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="W9" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="X9" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="10" spans="1:24">
@@ -4492,13 +4487,13 @@
         <v>120</v>
       </c>
       <c r="V10" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="W10" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="X10" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="11" spans="1:24">
@@ -4515,13 +4510,13 @@
         <v>12</v>
       </c>
       <c r="V11" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="W11" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="X11" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
     </row>
     <row r="12" spans="1:24">
@@ -4540,13 +4535,13 @@
       <c r="E12" s="10"/>
       <c r="F12" s="1"/>
       <c r="V12" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="W12" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="X12" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
     </row>
     <row r="13" spans="1:24">
@@ -4563,13 +4558,13 @@
         <v>12</v>
       </c>
       <c r="V13" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="W13" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="X13" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
     </row>
     <row r="14" spans="1:24">
@@ -4586,13 +4581,13 @@
         <v>12</v>
       </c>
       <c r="V14" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="W14" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="X14" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
     </row>
     <row r="15" spans="1:24">
@@ -4609,13 +4604,13 @@
         <v>12</v>
       </c>
       <c r="V15" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="W15" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="X15" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="16" spans="1:24">
@@ -4632,13 +4627,13 @@
         <v>12</v>
       </c>
       <c r="V16" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="W16" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="X16" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
     <row r="17" spans="1:24">
@@ -4655,13 +4650,13 @@
         <v>12</v>
       </c>
       <c r="V17" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="W17" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="X17" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
     </row>
     <row r="18" spans="1:24">
@@ -4678,13 +4673,13 @@
         <v>12</v>
       </c>
       <c r="V18" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="W18" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="X18" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
     </row>
     <row r="19" spans="1:24">
@@ -4701,13 +4696,13 @@
         <v>12</v>
       </c>
       <c r="V19" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="W19" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="X19" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
     </row>
     <row r="20" spans="1:24">
@@ -4724,13 +4719,13 @@
         <v>12</v>
       </c>
       <c r="V20" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="W20" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="X20" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
     </row>
     <row r="21" spans="1:24">
@@ -4747,13 +4742,13 @@
         <v>12</v>
       </c>
       <c r="V21" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="W21" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="X21" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
     </row>
     <row r="22" spans="1:24">
@@ -4770,13 +4765,13 @@
         <v>12</v>
       </c>
       <c r="V22" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="W22" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="X22" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
     </row>
     <row r="23" spans="1:24">
@@ -4793,10 +4788,10 @@
         <v>12</v>
       </c>
       <c r="V23" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="X23" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
     </row>
     <row r="24" spans="1:24">
@@ -4813,13 +4808,13 @@
         <v>12</v>
       </c>
       <c r="V24" t="s">
-        <v>485</v>
+        <v>481</v>
       </c>
       <c r="W24" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="X24" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
     </row>
     <row r="25" spans="1:24">
@@ -4836,13 +4831,13 @@
         <v>12</v>
       </c>
       <c r="V25" t="s">
-        <v>486</v>
+        <v>482</v>
       </c>
       <c r="W25" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="X25" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
     </row>
     <row r="26" spans="1:24">
@@ -4859,13 +4854,13 @@
         <v>71</v>
       </c>
       <c r="V26" t="s">
-        <v>487</v>
+        <v>483</v>
       </c>
       <c r="W26" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="X26" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
     </row>
     <row r="27" spans="1:24">
@@ -4882,13 +4877,13 @@
         <v>74</v>
       </c>
       <c r="V27" t="s">
-        <v>488</v>
+        <v>484</v>
       </c>
       <c r="W27" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="X27" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
     </row>
     <row r="28" spans="1:24">
@@ -4905,13 +4900,13 @@
         <v>74</v>
       </c>
       <c r="V28" t="s">
-        <v>489</v>
+        <v>485</v>
       </c>
       <c r="W28" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="X28" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
     </row>
     <row r="29" spans="1:24">
@@ -4928,13 +4923,13 @@
         <v>74</v>
       </c>
       <c r="V29" t="s">
-        <v>490</v>
+        <v>486</v>
       </c>
       <c r="W29" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="X29" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
     </row>
     <row r="30" spans="1:24">
@@ -4951,13 +4946,13 @@
         <v>74</v>
       </c>
       <c r="V30" t="s">
-        <v>491</v>
+        <v>487</v>
       </c>
       <c r="W30" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="X30" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="31" spans="1:24">
@@ -4971,13 +4966,13 @@
         <v>74</v>
       </c>
       <c r="V31" t="s">
-        <v>492</v>
+        <v>488</v>
       </c>
       <c r="W31" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="X31" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
     <row r="32" spans="1:24">
@@ -4991,13 +4986,13 @@
         <v>74</v>
       </c>
       <c r="V32" t="s">
-        <v>493</v>
+        <v>489</v>
       </c>
       <c r="W32" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="X32" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="33" spans="1:24">
@@ -5014,10 +5009,10 @@
         <v>12</v>
       </c>
       <c r="W33" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="X33" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
     </row>
     <row r="34" spans="1:24">
@@ -5034,10 +5029,10 @@
         <v>12</v>
       </c>
       <c r="W34" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="X34" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
     </row>
     <row r="35" spans="1:24">
@@ -5054,10 +5049,10 @@
         <v>12</v>
       </c>
       <c r="W35" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="X35" t="s">
-        <v>436</v>
+        <v>432</v>
       </c>
     </row>
     <row r="36" spans="1:24">
@@ -5074,10 +5069,10 @@
         <v>12</v>
       </c>
       <c r="W36" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="X36" t="s">
-        <v>437</v>
+        <v>433</v>
       </c>
     </row>
     <row r="37" spans="1:24">
@@ -5094,10 +5089,10 @@
         <v>12</v>
       </c>
       <c r="W37" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="X37" t="s">
-        <v>438</v>
+        <v>434</v>
       </c>
     </row>
     <row r="38" spans="1:24">
@@ -5114,10 +5109,10 @@
         <v>12</v>
       </c>
       <c r="W38" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="X38" t="s">
-        <v>439</v>
+        <v>435</v>
       </c>
     </row>
     <row r="39" spans="1:24">
@@ -5134,10 +5129,10 @@
         <v>12</v>
       </c>
       <c r="W39" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="X39" t="s">
-        <v>440</v>
+        <v>436</v>
       </c>
     </row>
     <row r="40" spans="1:24">
@@ -5145,13 +5140,13 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>368</v>
+        <v>364</v>
       </c>
       <c r="W40" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="X40" t="s">
-        <v>441</v>
+        <v>437</v>
       </c>
     </row>
     <row r="41" spans="1:24">
@@ -5162,10 +5157,10 @@
         <v>70</v>
       </c>
       <c r="W41" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="X41" t="s">
-        <v>442</v>
+        <v>438</v>
       </c>
     </row>
     <row r="42" spans="1:24">
@@ -5173,13 +5168,13 @@
         <v>76</v>
       </c>
       <c r="B42" t="s">
-        <v>369</v>
+        <v>365</v>
       </c>
       <c r="W42" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="X42" t="s">
-        <v>443</v>
+        <v>439</v>
       </c>
     </row>
     <row r="43" spans="1:24">
@@ -5187,10 +5182,10 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="X43" t="s">
-        <v>444</v>
+        <v>440</v>
       </c>
     </row>
     <row r="44" spans="1:24">
@@ -5198,296 +5193,296 @@
         <v>72</v>
       </c>
       <c r="B44" t="s">
-        <v>371</v>
+        <v>367</v>
       </c>
       <c r="W44" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="X44" t="s">
-        <v>445</v>
+        <v>441</v>
       </c>
     </row>
     <row r="45" spans="1:24">
       <c r="X45" t="s">
-        <v>446</v>
+        <v>442</v>
       </c>
     </row>
     <row r="46" spans="1:24">
       <c r="W46" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="X46" t="s">
-        <v>447</v>
+        <v>443</v>
       </c>
     </row>
     <row r="47" spans="1:24">
       <c r="W47" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="X47" t="s">
-        <v>448</v>
+        <v>444</v>
       </c>
     </row>
     <row r="48" spans="1:24">
       <c r="W48" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="X48" t="s">
-        <v>449</v>
+        <v>445</v>
       </c>
     </row>
     <row r="49" spans="1:24">
       <c r="W49" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="X49" t="s">
-        <v>450</v>
+        <v>446</v>
       </c>
     </row>
     <row r="50" spans="1:24">
       <c r="W50" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="X50" t="s">
-        <v>451</v>
+        <v>447</v>
       </c>
     </row>
     <row r="51" spans="1:24">
       <c r="W51" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="X51" t="s">
-        <v>452</v>
+        <v>448</v>
       </c>
     </row>
     <row r="52" spans="1:24">
       <c r="W52" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="X52" t="s">
-        <v>453</v>
+        <v>449</v>
       </c>
     </row>
     <row r="53" spans="1:24">
       <c r="W53" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="X53" t="s">
-        <v>454</v>
+        <v>450</v>
       </c>
     </row>
     <row r="54" spans="1:24">
       <c r="A54" s="1"/>
       <c r="W54" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
     </row>
     <row r="55" spans="1:24">
       <c r="W55" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
     </row>
     <row r="56" spans="1:24">
       <c r="W56" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
     </row>
     <row r="57" spans="1:24">
       <c r="W57" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
     </row>
     <row r="58" spans="1:24">
       <c r="W58" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
     </row>
     <row r="60" spans="1:24">
       <c r="W60" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
     </row>
     <row r="61" spans="1:24">
       <c r="W61" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="62" spans="1:24">
       <c r="W62" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="63" spans="1:24">
       <c r="W63" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="64" spans="1:24">
       <c r="W64" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="65" spans="23:23">
       <c r="W65" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
     </row>
     <row r="66" spans="23:23">
       <c r="W66" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
     </row>
     <row r="67" spans="23:23">
       <c r="W67" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
     </row>
     <row r="68" spans="23:23">
       <c r="W68" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="69" spans="23:23">
       <c r="W69" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
     </row>
     <row r="70" spans="23:23">
       <c r="W70" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
     </row>
     <row r="72" spans="23:23">
       <c r="W72" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
     </row>
     <row r="73" spans="23:23">
       <c r="W73" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
     </row>
     <row r="74" spans="23:23">
       <c r="W74" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="75" spans="23:23">
       <c r="W75" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
     </row>
     <row r="76" spans="23:23">
       <c r="W76" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="77" spans="23:23">
       <c r="W77" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="79" spans="23:23">
       <c r="W79" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="80" spans="23:23">
       <c r="W80" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="81" spans="23:23">
       <c r="W81" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="82" spans="23:23">
       <c r="W82" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
     </row>
     <row r="83" spans="23:23">
       <c r="W83" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
     </row>
     <row r="84" spans="23:23">
       <c r="W84" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
     </row>
     <row r="85" spans="23:23">
       <c r="W85" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
     </row>
     <row r="86" spans="23:23">
       <c r="W86" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="87" spans="23:23">
       <c r="W87" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="88" spans="23:23">
       <c r="W88" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
     <row r="90" spans="23:23">
       <c r="W90" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="91" spans="23:23">
       <c r="W91" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="93" spans="23:23">
       <c r="W93" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
     </row>
     <row r="94" spans="23:23">
       <c r="W94" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
     </row>
     <row r="95" spans="23:23">
       <c r="W95" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
     </row>
     <row r="96" spans="23:23">
       <c r="W96" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
     </row>
     <row r="105" spans="1:8">
       <c r="B105" t="s">
+        <v>201</v>
+      </c>
+      <c r="C105" t="s">
+        <v>202</v>
+      </c>
+      <c r="D105" t="s">
+        <v>203</v>
+      </c>
+      <c r="E105" t="s">
         <v>204</v>
       </c>
-      <c r="C105" t="s">
+      <c r="F105" t="s">
         <v>205</v>
       </c>
-      <c r="D105" t="s">
+      <c r="G105" t="s">
         <v>206</v>
       </c>
-      <c r="E105" t="s">
+      <c r="H105" t="s">
         <v>207</v>
-      </c>
-      <c r="F105" t="s">
-        <v>208</v>
-      </c>
-      <c r="G105" t="s">
-        <v>209</v>
-      </c>
-      <c r="H105" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -5495,13 +5490,13 @@
         <v>83</v>
       </c>
       <c r="B106" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C106" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D106" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -5509,13 +5504,13 @@
         <v>86</v>
       </c>
       <c r="B107" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C107" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="D107" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -5523,13 +5518,13 @@
         <v>89</v>
       </c>
       <c r="B108" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C108" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="D108" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
     </row>
     <row r="109" spans="1:8">
@@ -5537,13 +5532,13 @@
         <v>92</v>
       </c>
       <c r="B109" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C109" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="D109" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -5551,13 +5546,13 @@
         <v>93</v>
       </c>
       <c r="B110" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C110" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="D110" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -5565,13 +5560,13 @@
         <v>94</v>
       </c>
       <c r="B111" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="C111" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="D111" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -5579,13 +5574,13 @@
         <v>95</v>
       </c>
       <c r="B112" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="C112" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D112" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minor edits to the order of text in user guide
</commit_message>
<xml_diff>
--- a/templates/blank_context_template_sep2026.xlsx
+++ b/templates/blank_context_template_sep2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36DB2A15-C5BB-354B-846A-2C0480E630A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B75D44A-53BA-8B4E-B5A2-F17BBDCA3C50}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2480" yWindow="940" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2480" yWindow="940" windowWidth="32760" windowHeight="18640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Guide" sheetId="8" r:id="rId1"/>
@@ -2991,20 +2991,20 @@
         <v>167</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="68">
+    <row r="29" spans="1:4" ht="51">
       <c r="A29" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="68">
+      <c r="A30" s="15" t="s">
         <v>130</v>
       </c>
-      <c r="B29" s="16" t="s">
+      <c r="B30" s="16" t="s">
         <v>457</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="51">
-      <c r="A30" s="15" t="s">
-        <v>3</v>
-      </c>
-      <c r="B30" s="2" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="31" spans="1:4" ht="51">

</xml_diff>

<commit_message>
duplicate check for sample names added
</commit_message>
<xml_diff>
--- a/templates/blank_context_template_sep2026.xlsx
+++ b/templates/blank_context_template_sep2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF1444BF-CB54-3540-AFFD-E7551C377C72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{179EA4FC-FAC2-7945-8B72-0B6003398549}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4680" yWindow="940" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2209,14 +2209,14 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2431,7 +2431,17 @@
     <cellStyle name="Hyperlink" xfId="199" builtinId="8" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2797,19 +2807,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="83" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="49" t="s">
         <v>150</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
+      <c r="B1" s="49"/>
+      <c r="C1" s="49"/>
       <c r="D1" s="45"/>
     </row>
     <row r="2" spans="1:4" s="8" customFormat="1" ht="148" customHeight="1">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="48" t="s">
         <v>199</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
+      <c r="B2" s="48"/>
+      <c r="C2" s="48"/>
       <c r="D2" s="26"/>
     </row>
     <row r="5" spans="1:4" ht="19">
@@ -3298,10 +3308,10 @@
       <c r="R1" s="43"/>
       <c r="S1" s="43"/>
       <c r="T1" s="43"/>
-      <c r="U1" s="49" t="s">
+      <c r="U1" s="47" t="s">
         <v>133</v>
       </c>
-      <c r="V1" s="49"/>
+      <c r="V1" s="47"/>
       <c r="W1" s="24"/>
       <c r="X1" s="24"/>
       <c r="Y1" s="25"/>
@@ -3474,13 +3484,16 @@
     <mergeCell ref="U1:V1"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
+  <conditionalFormatting sqref="B4:B1048576">
+    <cfRule type="duplicateValues" dxfId="0" priority="1"/>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="expression" priority="1" id="{7C4831EF-860F-7B4C-96B3-F4D36BC0BBA8}">
+          <x14:cfRule type="expression" priority="2" id="{7C4831EF-860F-7B4C-96B3-F4D36BC0BBA8}">
             <xm:f>AND(D4&lt;&gt;"",COUNTIF(Sites!$A$3:$A$1048576,D4)=0)</xm:f>
             <x14:dxf>
               <font>
@@ -3918,7 +3931,7 @@
     <sortCondition ref="A2:A61"/>
   </sortState>
   <conditionalFormatting sqref="A2:A61">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="1" priority="2"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <extLst>

</xml_diff>

<commit_message>
added validation to columns
</commit_message>
<xml_diff>
--- a/templates/blank_context_template_sep2026.xlsx
+++ b/templates/blank_context_template_sep2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6850174E-A864-9D46-B66A-6B220FA12E2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075FBBD6-6F49-D745-A1D3-4FAE6018BDF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1540" yWindow="600" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="600" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Guide" sheetId="8" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Samples" sheetId="2" r:id="rId4"/>
     <sheet name="PrepMethods" sheetId="10" r:id="rId5"/>
     <sheet name="Dictionary of Sed Structures" sheetId="9" r:id="rId6"/>
-    <sheet name="Dropdowns" sheetId="7" state="hidden" r:id="rId7"/>
+    <sheet name="Dropdowns" sheetId="7" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="606" uniqueCount="510">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="513">
   <si>
     <t>lith_comp</t>
   </si>
@@ -1806,6 +1806,15 @@
   </si>
   <si>
     <t>if multiple use full names, comma-separated list</t>
+  </si>
+  <si>
+    <t>Boolean</t>
+  </si>
+  <si>
+    <t>t</t>
+  </si>
+  <si>
+    <t>f</t>
   </si>
 </sst>
 </file>
@@ -2206,7 +2215,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="60">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2255,20 +2264,8 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2282,20 +2279,29 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2306,19 +2312,15 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="13" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="201">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
@@ -2908,17 +2910,17 @@
     <col min="4" max="4" width="58" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="52" customFormat="1" ht="83" customHeight="1">
-      <c r="A1" s="51" t="s">
+    <row r="1" spans="1:4" s="42" customFormat="1" ht="83" customHeight="1">
+      <c r="A1" s="41" t="s">
         <v>500</v>
       </c>
-      <c r="B1" s="51"/>
+      <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:4" s="8" customFormat="1" ht="158" customHeight="1">
-      <c r="A2" s="47" t="s">
+      <c r="A2" s="49" t="s">
         <v>507</v>
       </c>
-      <c r="B2" s="47"/>
+      <c r="B2" s="49"/>
       <c r="C2" s="26"/>
       <c r="D2" s="26"/>
     </row>
@@ -2926,25 +2928,25 @@
       <c r="A4" s="9" t="s">
         <v>508</v>
       </c>
-      <c r="B4" s="53"/>
-    </row>
-    <row r="5" spans="1:4" s="55" customFormat="1" ht="19">
-      <c r="A5" s="54"/>
-    </row>
-    <row r="6" spans="1:4" s="55" customFormat="1" ht="19">
-      <c r="A6" s="54"/>
-    </row>
-    <row r="7" spans="1:4" s="55" customFormat="1" ht="19">
-      <c r="A7" s="54"/>
-    </row>
-    <row r="8" spans="1:4" s="55" customFormat="1" ht="19">
-      <c r="A8" s="54"/>
+      <c r="B4" s="43"/>
+    </row>
+    <row r="5" spans="1:4" ht="19">
+      <c r="A5" s="44"/>
+    </row>
+    <row r="6" spans="1:4" ht="19">
+      <c r="A6" s="44"/>
+    </row>
+    <row r="7" spans="1:4" ht="19">
+      <c r="A7" s="44"/>
+    </row>
+    <row r="8" spans="1:4" ht="19">
+      <c r="A8" s="44"/>
     </row>
     <row r="11" spans="1:4" ht="19">
       <c r="A11" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="B11" s="53"/>
+      <c r="B11" s="43"/>
     </row>
     <row r="12" spans="1:4" ht="51">
       <c r="A12" s="7" t="s">
@@ -3030,7 +3032,7 @@
       <c r="A24" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="B24" s="53"/>
+      <c r="B24" s="43"/>
     </row>
     <row r="25" spans="1:3" ht="34">
       <c r="A25" s="15" t="s">
@@ -3160,7 +3162,7 @@
       <c r="A41" s="9" t="s">
         <v>360</v>
       </c>
-      <c r="B41" s="53"/>
+      <c r="B41" s="43"/>
     </row>
     <row r="42" spans="1:4" ht="102">
       <c r="A42" s="15" t="s">
@@ -3202,42 +3204,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="45" t="s">
         <v>495</v>
       </c>
-      <c r="B1" s="57">
+      <c r="B1" s="46">
         <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:3">
-      <c r="A2" s="56" t="s">
+      <c r="A2" s="45" t="s">
         <v>496</v>
       </c>
-      <c r="B2" s="58">
+      <c r="B2" s="47">
         <v>46283</v>
       </c>
     </row>
     <row r="3" spans="1:3">
-      <c r="A3" s="56" t="s">
+      <c r="A3" s="45" t="s">
         <v>497</v>
       </c>
-      <c r="B3" s="59" t="s">
+      <c r="B3" s="48" t="s">
         <v>501</v>
       </c>
     </row>
     <row r="4" spans="1:3">
-      <c r="A4" s="56" t="s">
+      <c r="A4" s="45" t="s">
         <v>498</v>
       </c>
-      <c r="B4" s="59" t="s">
+      <c r="B4" s="48" t="s">
         <v>503</v>
       </c>
     </row>
     <row r="5" spans="1:3">
-      <c r="A5" s="56" t="s">
+      <c r="A5" s="45" t="s">
         <v>499</v>
       </c>
-      <c r="B5" s="59" t="s">
+      <c r="B5" s="48" t="s">
         <v>502</v>
       </c>
     </row>
@@ -3397,16 +3399,16 @@
     </row>
     <row r="3" spans="1:19">
       <c r="A3" s="27"/>
-      <c r="G3" s="35"/>
-      <c r="H3" s="35"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
     </row>
     <row r="4" spans="1:19">
       <c r="A4" s="27"/>
-      <c r="G4" s="35"/>
-      <c r="H4" s="35"/>
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
     </row>
     <row r="5" spans="1:19">
-      <c r="H5" s="36"/>
+      <c r="H5" s="32"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A1048576">
@@ -3456,10 +3458,10 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
-    <col min="2" max="2" width="23.6640625" style="45" customWidth="1"/>
-    <col min="3" max="3" width="38.33203125" customWidth="1"/>
-    <col min="4" max="4" width="44" customWidth="1"/>
-    <col min="5" max="5" width="29.5" customWidth="1"/>
+    <col min="2" max="2" width="23.6640625" style="40" customWidth="1"/>
+    <col min="3" max="3" width="36.83203125" customWidth="1"/>
+    <col min="4" max="4" width="44.5" customWidth="1"/>
+    <col min="5" max="5" width="27" customWidth="1"/>
     <col min="6" max="6" width="29.33203125" customWidth="1"/>
     <col min="7" max="8" width="29.6640625" customWidth="1"/>
     <col min="9" max="9" width="34" customWidth="1"/>
@@ -3484,48 +3486,48 @@
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
       <c r="E1" s="14"/>
-      <c r="F1" s="42" t="s">
+      <c r="F1" s="37" t="s">
         <v>126</v>
       </c>
-      <c r="G1" s="42"/>
-      <c r="H1" s="42"/>
-      <c r="I1" s="42"/>
-      <c r="J1" s="42"/>
-      <c r="K1" s="42"/>
-      <c r="L1" s="42"/>
-      <c r="M1" s="43" t="s">
+      <c r="G1" s="37"/>
+      <c r="H1" s="37"/>
+      <c r="I1" s="37"/>
+      <c r="J1" s="37"/>
+      <c r="K1" s="37"/>
+      <c r="L1" s="37"/>
+      <c r="M1" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="N1" s="43"/>
-      <c r="O1" s="43"/>
-      <c r="P1" s="43"/>
-      <c r="Q1" s="43"/>
-      <c r="R1" s="43"/>
-      <c r="S1" s="43"/>
-      <c r="T1" s="43"/>
-      <c r="U1" s="46" t="s">
+      <c r="N1" s="38"/>
+      <c r="O1" s="38"/>
+      <c r="P1" s="38"/>
+      <c r="Q1" s="38"/>
+      <c r="R1" s="38"/>
+      <c r="S1" s="38"/>
+      <c r="T1" s="38"/>
+      <c r="U1" s="50" t="s">
         <v>133</v>
       </c>
-      <c r="V1" s="46"/>
+      <c r="V1" s="50"/>
       <c r="W1" s="24"/>
       <c r="X1" s="24"/>
       <c r="Y1" s="25"/>
       <c r="Z1" s="25"/>
     </row>
     <row r="2" spans="1:27" s="1" customFormat="1" ht="30" customHeight="1">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="30" t="s">
         <v>256</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="54" t="s">
         <v>187</v>
       </c>
-      <c r="C2" s="30" t="s">
+      <c r="C2" s="55" t="s">
         <v>188</v>
       </c>
-      <c r="D2" s="29" t="s">
+      <c r="D2" s="55" t="s">
         <v>189</v>
       </c>
-      <c r="E2" s="29" t="s">
+      <c r="E2" s="55" t="s">
         <v>255</v>
       </c>
       <c r="F2" s="11" t="s">
@@ -3534,7 +3536,7 @@
       <c r="G2" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="H2" s="32" t="s">
+      <c r="H2" s="29" t="s">
         <v>328</v>
       </c>
       <c r="I2" s="11" t="s">
@@ -3599,16 +3601,16 @@
       <c r="A3" s="21" t="s">
         <v>468</v>
       </c>
-      <c r="B3" s="40" t="s">
+      <c r="B3" s="36" t="s">
         <v>467</v>
       </c>
-      <c r="C3" s="41" t="s">
+      <c r="C3" s="36" t="s">
         <v>366</v>
       </c>
-      <c r="D3" s="40" t="s">
+      <c r="D3" s="36" t="s">
         <v>489</v>
       </c>
-      <c r="E3" s="33" t="s">
+      <c r="E3" s="56" t="s">
         <v>156</v>
       </c>
       <c r="F3" s="3" t="s">
@@ -3680,7 +3682,7 @@
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <conditionalFormatting sqref="B4:B1048576">
-    <cfRule type="duplicateValues" dxfId="1" priority="1"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292"/>
@@ -3706,7 +3708,7 @@
       </x14:conditionalFormattings>
     </ext>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="7">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="8">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{00000000-0002-0000-0200-000001000000}">
           <x14:formula1>
             <xm:f>Dropdowns!$F$3:$F$6</xm:f>
@@ -3749,6 +3751,12 @@
           </x14:formula1>
           <xm:sqref>D4:D1048576</xm:sqref>
         </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showDropDown="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4CE48C8C-9526-784E-8824-0DD17C105F93}">
+          <x14:formula1>
+            <xm:f>Dropdowns!$Y$2:$Y$3</xm:f>
+          </x14:formula1>
+          <xm:sqref>Q4:Q1048576 J4:J1048576</xm:sqref>
+        </x14:dataValidation>
       </x14:dataValidations>
     </ext>
     <ext xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" uri="{64002731-A6B0-56B0-2670-7721B7C09600}">
@@ -3769,7 +3777,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="33" t="s">
         <v>456</v>
       </c>
       <c r="B1" s="12" t="s">
@@ -3780,10 +3788,10 @@
       </c>
     </row>
     <row r="2" spans="1:3" s="16" customFormat="1" ht="35" customHeight="1">
-      <c r="A2" s="38" t="s">
+      <c r="A2" s="34" t="s">
         <v>466</v>
       </c>
-      <c r="B2" s="39" t="s">
+      <c r="B2" s="35" t="s">
         <v>469</v>
       </c>
       <c r="C2" s="7" t="s">
@@ -3816,7 +3824,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="26" customHeight="1">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="39" t="s">
         <v>41</v>
       </c>
       <c r="B1" s="22"/>
@@ -4139,7 +4147,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:X112"/>
+  <dimension ref="A1:Y112"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="19.1640625" customWidth="1"/>
@@ -4163,23 +4171,23 @@
     <col min="24" max="24" width="22.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24">
-      <c r="A1" s="48" t="s">
+    <row r="1" spans="1:25">
+      <c r="A1" s="51" t="s">
         <v>227</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
+      <c r="B1" s="51"/>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
       <c r="E1" s="14" t="s">
         <v>228</v>
       </c>
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
-      <c r="H1" s="49" t="s">
+      <c r="H1" s="52" t="s">
         <v>229</v>
       </c>
-      <c r="I1" s="49"/>
-      <c r="J1" s="49"/>
+      <c r="I1" s="52"/>
+      <c r="J1" s="52"/>
       <c r="K1" s="5" t="s">
         <v>230</v>
       </c>
@@ -4187,29 +4195,32 @@
       <c r="M1" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="N1" s="50" t="s">
+      <c r="N1" s="53" t="s">
         <v>262</v>
       </c>
-      <c r="O1" s="50"/>
-      <c r="P1" s="50"/>
-      <c r="Q1" s="50"/>
-      <c r="R1" s="50"/>
-      <c r="S1" s="48" t="s">
+      <c r="O1" s="53"/>
+      <c r="P1" s="53"/>
+      <c r="Q1" s="53"/>
+      <c r="R1" s="53"/>
+      <c r="S1" s="51" t="s">
         <v>142</v>
       </c>
-      <c r="T1" s="48"/>
-      <c r="U1" s="48"/>
+      <c r="T1" s="51"/>
+      <c r="U1" s="51"/>
       <c r="V1" s="19" t="s">
         <v>239</v>
       </c>
-      <c r="W1" s="31" t="s">
+      <c r="W1" s="28" t="s">
         <v>264</v>
       </c>
       <c r="X1" s="4" t="s">
         <v>449</v>
       </c>
-    </row>
-    <row r="2" spans="1:24">
+      <c r="Y1" t="s">
+        <v>510</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -4258,8 +4269,11 @@
       <c r="X2" t="s">
         <v>450</v>
       </c>
-    </row>
-    <row r="3" spans="1:24">
+      <c r="Y2" t="s">
+        <v>511</v>
+      </c>
+    </row>
+    <row r="3" spans="1:25">
       <c r="A3">
         <v>1</v>
       </c>
@@ -4323,8 +4337,11 @@
       <c r="X3" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="4" spans="1:24">
+      <c r="Y3" t="s">
+        <v>512</v>
+      </c>
+    </row>
+    <row r="4" spans="1:25">
       <c r="A4">
         <v>2</v>
       </c>
@@ -4389,7 +4406,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="5" spans="1:24">
+    <row r="5" spans="1:25">
       <c r="A5">
         <v>3</v>
       </c>
@@ -4454,7 +4471,7 @@
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:24">
+    <row r="6" spans="1:25">
       <c r="A6">
         <v>4</v>
       </c>
@@ -4507,7 +4524,7 @@
         <v>401</v>
       </c>
     </row>
-    <row r="7" spans="1:24">
+    <row r="7" spans="1:25">
       <c r="A7">
         <v>5</v>
       </c>
@@ -4551,7 +4568,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="8" spans="1:24">
+    <row r="8" spans="1:25">
       <c r="A8">
         <v>6</v>
       </c>
@@ -4595,7 +4612,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="9" spans="1:24">
+    <row r="9" spans="1:25">
       <c r="A9">
         <v>7</v>
       </c>
@@ -4630,7 +4647,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="10" spans="1:24">
+    <row r="10" spans="1:25">
       <c r="A10">
         <v>8</v>
       </c>
@@ -4659,7 +4676,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="11" spans="1:24">
+    <row r="11" spans="1:25">
       <c r="A11">
         <v>9</v>
       </c>
@@ -4682,7 +4699,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="12" spans="1:24">
+    <row r="12" spans="1:25">
       <c r="A12">
         <v>10</v>
       </c>
@@ -4707,7 +4724,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:25">
       <c r="A13">
         <v>11</v>
       </c>
@@ -4730,7 +4747,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:25">
       <c r="A14">
         <v>12</v>
       </c>
@@ -4753,7 +4770,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:25">
       <c r="A15">
         <v>13</v>
       </c>
@@ -4776,7 +4793,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:25">
       <c r="A16">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
changed meta bin text
</commit_message>
<xml_diff>
--- a/templates/blank_context_template_sep2026.xlsx
+++ b/templates/blank_context_template_sep2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10914"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10920"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{075FBBD6-6F49-D745-A1D3-4FAE6018BDF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8CF96E4-687F-4048-9F68-F5C3FB9707A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4680" yWindow="600" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="600" windowWidth="32760" windowHeight="18640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="User Guide" sheetId="8" r:id="rId1"/>
@@ -493,13 +493,6 @@
   </si>
   <si>
     <t>Diagenetic zone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sites are sorted into three low-grade metamorphic bins, roughly based on metapelite zones as follows: 
-1) Diagenetic zone. Under mature, preserved biomarkers, KI&gt;0.42, CAI ≤3, Ro &lt;2.0, facies: zeolite-subgreenschist facies, grade: diagenesis-very low grade 
-2) Anchizone. Over-mature, no preserved biomarkers, CAI=4, Ro 2-4, facies: sub-greenschist, grade: very low grade 
-3) Epizone. Ro&gt;4, CAI=5, KI&lt;0.25, facies: greenschist, grade: low-grade
-</t>
   </si>
   <si>
     <t>env_id</t>
@@ -1815,6 +1808,13 @@
   </si>
   <si>
     <t>f</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sites are sorted into three low-grade metamorphic bins, roughly based on metapelite zones as follows: 
+1) Diagenetic zone. Under mature to post-mature (up to wet gas and condensate window), biomarkers may be preserved, KI&gt;0.42, CAI ≤3, Ro &lt;2.0, facies: zeolite-subgreenschist facies, grade: diagenesis-very low grade
+2) Anchizone. Over-mature, no preserved biomarkers, CAI=4, Ro 2-4, facies: sub-greenschist, grade: very low grade 
+3) Epizone. Ro&gt;4, CAI=5, KI&lt;0.25, facies: greenschist, grade: low-grade
+</t>
   </si>
 </sst>
 </file>
@@ -2297,11 +2297,20 @@
     <xf numFmtId="164" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="14" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="14" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2311,15 +2320,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="201">
@@ -2912,21 +2912,21 @@
   <sheetData>
     <row r="1" spans="1:4" s="42" customFormat="1" ht="83" customHeight="1">
       <c r="A1" s="41" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B1" s="41"/>
     </row>
     <row r="2" spans="1:4" s="8" customFormat="1" ht="158" customHeight="1">
-      <c r="A2" s="49" t="s">
-        <v>507</v>
-      </c>
-      <c r="B2" s="49"/>
+      <c r="A2" s="53" t="s">
+        <v>506</v>
+      </c>
+      <c r="B2" s="53"/>
       <c r="C2" s="26"/>
       <c r="D2" s="26"/>
     </row>
     <row r="4" spans="1:4" ht="19">
       <c r="A4" s="9" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="B4" s="43"/>
     </row>
@@ -2953,7 +2953,7 @@
         <v>114</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="68">
@@ -2961,7 +2961,7 @@
         <v>140</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="51">
@@ -2969,7 +2969,7 @@
         <v>139</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="34">
@@ -2977,7 +2977,7 @@
         <v>105</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="34">
@@ -2985,23 +2985,23 @@
         <v>117</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:3" ht="34">
       <c r="A17" s="7" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="170">
       <c r="A18" s="7" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>151</v>
+        <v>512</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="68">
@@ -3009,7 +3009,7 @@
         <v>106</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
     </row>
     <row r="20" spans="1:3" ht="51">
@@ -3017,7 +3017,7 @@
         <v>138</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
     </row>
     <row r="21" spans="1:3">
@@ -3025,7 +3025,7 @@
         <v>115</v>
       </c>
       <c r="B21" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
     </row>
     <row r="24" spans="1:3" ht="19">
@@ -3039,32 +3039,32 @@
         <v>124</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="170">
       <c r="A26" s="15" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B26" s="16" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
     </row>
     <row r="27" spans="1:3" ht="409.6">
       <c r="A27" s="15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="C27" s="7"/>
     </row>
     <row r="28" spans="1:3" ht="68">
       <c r="A28" s="15" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C28" s="7"/>
     </row>
@@ -3073,7 +3073,7 @@
         <v>125</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
     <row r="30" spans="1:3" ht="51">
@@ -3081,7 +3081,7 @@
         <v>136</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
     </row>
     <row r="31" spans="1:3">
@@ -3097,7 +3097,7 @@
         <v>127</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C32" s="6"/>
     </row>
@@ -3106,7 +3106,7 @@
         <v>134</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="34" spans="1:4" ht="51">
@@ -3114,7 +3114,7 @@
         <v>129</v>
       </c>
       <c r="B34" s="16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="35" spans="1:4" ht="51">
@@ -3122,7 +3122,7 @@
         <v>3</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="36" spans="1:4" ht="68">
@@ -3130,7 +3130,7 @@
         <v>130</v>
       </c>
       <c r="B36" s="16" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
     </row>
     <row r="37" spans="1:4" ht="51">
@@ -3138,16 +3138,16 @@
         <v>133</v>
       </c>
       <c r="B37" s="16" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="D37" s="2"/>
     </row>
     <row r="38" spans="1:4" ht="187">
       <c r="A38" s="15" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B38" s="16" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="39" spans="1:4" ht="51">
@@ -3155,29 +3155,29 @@
         <v>115</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="41" spans="1:4" ht="19">
       <c r="A41" s="9" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="B41" s="43"/>
     </row>
     <row r="42" spans="1:4" ht="102">
       <c r="A42" s="15" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B42" s="16" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
     </row>
     <row r="43" spans="1:4" ht="51">
       <c r="A43" s="15" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
   </sheetData>
@@ -3205,7 +3205,7 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="45" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="B1" s="46">
         <v>2</v>
@@ -3213,7 +3213,7 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" s="45" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B2" s="47">
         <v>46283</v>
@@ -3221,44 +3221,44 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" s="45" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="B3" s="48" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" s="45" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="B4" s="48" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" s="45" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="B5" s="48" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" s="1" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C7" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" s="1" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" s="1" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
   </sheetData>
@@ -3291,10 +3291,10 @@
   <sheetData>
     <row r="1" spans="1:19" s="1" customFormat="1" ht="38" customHeight="1">
       <c r="A1" s="12" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="C1" s="17" t="s">
         <v>111</v>
@@ -3309,10 +3309,10 @@
         <v>114</v>
       </c>
       <c r="G1" s="17" t="s">
+        <v>195</v>
+      </c>
+      <c r="H1" s="17" t="s">
         <v>196</v>
-      </c>
-      <c r="H1" s="17" t="s">
-        <v>197</v>
       </c>
       <c r="I1" s="17" t="s">
         <v>139</v>
@@ -3321,7 +3321,7 @@
         <v>123</v>
       </c>
       <c r="K1" s="11" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="L1" s="13" t="s">
         <v>117</v>
@@ -3330,7 +3330,7 @@
         <v>116</v>
       </c>
       <c r="N1" s="18" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="O1" s="20" t="s">
         <v>131</v>
@@ -3342,7 +3342,7 @@
         <v>106</v>
       </c>
       <c r="R1" s="20" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="S1" s="1" t="s">
         <v>115</v>
@@ -3351,50 +3351,50 @@
     <row r="2" spans="1:19">
       <c r="A2" s="4"/>
       <c r="B2" s="14" t="s">
+        <v>172</v>
+      </c>
+      <c r="C2" s="14" t="s">
         <v>173</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="D2" s="14" t="s">
         <v>174</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="E2" s="14" t="s">
         <v>175</v>
       </c>
-      <c r="E2" s="14" t="s">
+      <c r="F2" s="14" t="s">
         <v>176</v>
-      </c>
-      <c r="F2" s="14" t="s">
-        <v>177</v>
       </c>
       <c r="G2" s="14"/>
       <c r="H2" s="14"/>
       <c r="I2" s="14" t="s">
+        <v>177</v>
+      </c>
+      <c r="J2" s="14" t="s">
+        <v>459</v>
+      </c>
+      <c r="K2" s="3" t="s">
         <v>178</v>
       </c>
-      <c r="J2" s="14" t="s">
-        <v>460</v>
-      </c>
-      <c r="K2" s="3" t="s">
+      <c r="L2" s="5" t="s">
         <v>179</v>
       </c>
-      <c r="L2" s="5" t="s">
+      <c r="M2" s="5" t="s">
         <v>180</v>
       </c>
-      <c r="M2" s="5" t="s">
-        <v>181</v>
-      </c>
       <c r="N2" s="19" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="O2" s="21"/>
       <c r="P2" s="21"/>
       <c r="Q2" s="21" t="s">
+        <v>460</v>
+      </c>
+      <c r="R2" s="21" t="s">
         <v>461</v>
       </c>
-      <c r="R2" s="21" t="s">
-        <v>462</v>
-      </c>
       <c r="S2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="3" spans="1:19">
@@ -3505,10 +3505,10 @@
       <c r="R1" s="38"/>
       <c r="S1" s="38"/>
       <c r="T1" s="38"/>
-      <c r="U1" s="50" t="s">
+      <c r="U1" s="52" t="s">
         <v>133</v>
       </c>
-      <c r="V1" s="50"/>
+      <c r="V1" s="52"/>
       <c r="W1" s="24"/>
       <c r="X1" s="24"/>
       <c r="Y1" s="25"/>
@@ -3516,55 +3516,55 @@
     </row>
     <row r="2" spans="1:27" s="1" customFormat="1" ht="30" customHeight="1">
       <c r="A2" s="30" t="s">
-        <v>256</v>
-      </c>
-      <c r="B2" s="54" t="s">
+        <v>255</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>186</v>
+      </c>
+      <c r="C2" s="50" t="s">
         <v>187</v>
       </c>
-      <c r="C2" s="55" t="s">
+      <c r="D2" s="50" t="s">
         <v>188</v>
       </c>
-      <c r="D2" s="55" t="s">
+      <c r="E2" s="50" t="s">
+        <v>254</v>
+      </c>
+      <c r="F2" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="E2" s="55" t="s">
-        <v>255</v>
-      </c>
-      <c r="F2" s="11" t="s">
+      <c r="G2" s="11" t="s">
         <v>190</v>
       </c>
-      <c r="G2" s="11" t="s">
-        <v>191</v>
-      </c>
       <c r="H2" s="29" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="I2" s="11" t="s">
         <v>125</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K2" s="11" t="s">
         <v>108</v>
       </c>
       <c r="L2" s="11" t="s">
+        <v>191</v>
+      </c>
+      <c r="M2" s="12" t="s">
         <v>192</v>
       </c>
-      <c r="M2" s="12" t="s">
-        <v>193</v>
-      </c>
       <c r="N2" s="12" t="s">
+        <v>182</v>
+      </c>
+      <c r="O2" s="12" t="s">
         <v>183</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="P2" s="12" t="s">
         <v>184</v>
       </c>
-      <c r="P2" s="12" t="s">
-        <v>185</v>
-      </c>
       <c r="Q2" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="R2" s="12" t="s">
         <v>3</v>
@@ -3576,22 +3576,22 @@
         <v>129</v>
       </c>
       <c r="U2" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="V2" s="13" t="s">
         <v>194</v>
       </c>
-      <c r="V2" s="13" t="s">
-        <v>195</v>
-      </c>
       <c r="W2" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="X2" s="13" t="s">
+        <v>230</v>
+      </c>
+      <c r="Y2" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="Z2" s="20" t="s">
         <v>232</v>
-      </c>
-      <c r="X2" s="13" t="s">
-        <v>231</v>
-      </c>
-      <c r="Y2" s="20" t="s">
-        <v>329</v>
-      </c>
-      <c r="Z2" s="20" t="s">
-        <v>233</v>
       </c>
       <c r="AA2" s="1" t="s">
         <v>115</v>
@@ -3599,81 +3599,81 @@
     </row>
     <row r="3" spans="1:27" ht="17">
       <c r="A3" s="21" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="B3" s="36" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="C3" s="36" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D3" s="36" t="s">
-        <v>489</v>
-      </c>
-      <c r="E3" s="56" t="s">
+        <v>488</v>
+      </c>
+      <c r="E3" s="51" t="s">
+        <v>155</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>156</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>157</v>
-      </c>
       <c r="G3" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="M3" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="O3" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P3" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="Q3" s="4"/>
       <c r="R3" s="4" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="S3" s="4" t="s">
+        <v>366</v>
+      </c>
+      <c r="T3" s="4" t="s">
         <v>367</v>
       </c>
-      <c r="T3" s="4" t="s">
-        <v>368</v>
-      </c>
       <c r="U3" s="5" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="V3" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="X3" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="Y3" s="21" t="s">
+        <v>464</v>
+      </c>
+      <c r="Z3" s="21" t="s">
         <v>463</v>
       </c>
-      <c r="W3" s="5" t="s">
-        <v>460</v>
-      </c>
-      <c r="X3" s="5" t="s">
-        <v>460</v>
-      </c>
-      <c r="Y3" s="21" t="s">
-        <v>465</v>
-      </c>
-      <c r="Z3" s="21" t="s">
-        <v>464</v>
-      </c>
       <c r="AA3" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
   </sheetData>
@@ -3778,10 +3778,10 @@
   <sheetData>
     <row r="1" spans="1:3">
       <c r="A1" s="33" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="B1" s="12" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>115</v>
@@ -3789,13 +3789,13 @@
     </row>
     <row r="2" spans="1:3" s="16" customFormat="1" ht="35" customHeight="1">
       <c r="A2" s="34" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="B2" s="35" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
     </row>
   </sheetData>
@@ -3831,7 +3831,7 @@
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>386</v>
+        <v>385</v>
       </c>
     </row>
     <row r="3" spans="1:2">
@@ -3846,7 +3846,7 @@
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>396</v>
+        <v>395</v>
       </c>
     </row>
     <row r="6" spans="1:2">
@@ -3901,7 +3901,7 @@
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>395</v>
+        <v>394</v>
       </c>
     </row>
     <row r="17" spans="1:1">
@@ -3911,7 +3911,7 @@
     </row>
     <row r="18" spans="1:1">
       <c r="A18" t="s">
-        <v>390</v>
+        <v>389</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -3926,7 +3926,7 @@
     </row>
     <row r="21" spans="1:1">
       <c r="A21" t="s">
-        <v>384</v>
+        <v>383</v>
       </c>
     </row>
     <row r="22" spans="1:1">
@@ -3951,22 +3951,22 @@
     </row>
     <row r="26" spans="1:1">
       <c r="A26" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
     </row>
     <row r="27" spans="1:1">
       <c r="A27" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" t="s">
-        <v>378</v>
+        <v>377</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" t="s">
-        <v>370</v>
+        <v>369</v>
       </c>
     </row>
     <row r="30" spans="1:1">
@@ -3981,7 +3981,7 @@
     </row>
     <row r="32" spans="1:1">
       <c r="A32" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
     </row>
     <row r="33" spans="1:1">
@@ -3991,22 +3991,22 @@
     </row>
     <row r="34" spans="1:1">
       <c r="A34" t="s">
-        <v>385</v>
+        <v>384</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" t="s">
-        <v>383</v>
+        <v>382</v>
       </c>
     </row>
     <row r="38" spans="1:1">
@@ -4021,7 +4021,7 @@
     </row>
     <row r="40" spans="1:1">
       <c r="A40" t="s">
-        <v>392</v>
+        <v>391</v>
       </c>
     </row>
     <row r="41" spans="1:1">
@@ -4036,22 +4036,22 @@
     </row>
     <row r="43" spans="1:1">
       <c r="A43" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" t="s">
-        <v>381</v>
+        <v>380</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="47" spans="1:1">
@@ -4061,12 +4061,12 @@
     </row>
     <row r="48" spans="1:1">
       <c r="A48" t="s">
-        <v>397</v>
+        <v>396</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" t="s">
-        <v>387</v>
+        <v>386</v>
       </c>
     </row>
     <row r="50" spans="1:1">
@@ -4076,22 +4076,22 @@
     </row>
     <row r="51" spans="1:1">
       <c r="A51" t="s">
-        <v>371</v>
+        <v>370</v>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" t="s">
-        <v>389</v>
+        <v>388</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" t="s">
-        <v>394</v>
+        <v>393</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" t="s">
-        <v>391</v>
+        <v>390</v>
       </c>
     </row>
     <row r="55" spans="1:1">
@@ -4106,7 +4106,7 @@
     </row>
     <row r="57" spans="1:1">
       <c r="A57" t="s">
-        <v>393</v>
+        <v>392</v>
       </c>
     </row>
     <row r="58" spans="1:1">
@@ -4116,17 +4116,17 @@
     </row>
     <row r="59" spans="1:1">
       <c r="A59" t="s">
-        <v>388</v>
+        <v>387</v>
       </c>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" t="s">
-        <v>382</v>
+        <v>381</v>
       </c>
     </row>
     <row r="61" spans="1:1">
       <c r="A61" t="s">
-        <v>380</v>
+        <v>379</v>
       </c>
     </row>
   </sheetData>
@@ -4172,52 +4172,52 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="54" t="s">
+        <v>226</v>
+      </c>
+      <c r="B1" s="54"/>
+      <c r="C1" s="54"/>
+      <c r="D1" s="54"/>
+      <c r="E1" s="14" t="s">
         <v>227</v>
-      </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="14" t="s">
-        <v>228</v>
       </c>
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
-      <c r="H1" s="52" t="s">
+      <c r="H1" s="55" t="s">
+        <v>228</v>
+      </c>
+      <c r="I1" s="55"/>
+      <c r="J1" s="55"/>
+      <c r="K1" s="5" t="s">
         <v>229</v>
-      </c>
-      <c r="I1" s="52"/>
-      <c r="J1" s="52"/>
-      <c r="K1" s="5" t="s">
-        <v>230</v>
       </c>
       <c r="L1" s="5"/>
       <c r="M1" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="N1" s="53" t="s">
-        <v>262</v>
-      </c>
-      <c r="O1" s="53"/>
-      <c r="P1" s="53"/>
-      <c r="Q1" s="53"/>
-      <c r="R1" s="53"/>
-      <c r="S1" s="51" t="s">
+      <c r="N1" s="56" t="s">
+        <v>261</v>
+      </c>
+      <c r="O1" s="56"/>
+      <c r="P1" s="56"/>
+      <c r="Q1" s="56"/>
+      <c r="R1" s="56"/>
+      <c r="S1" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="T1" s="51"/>
-      <c r="U1" s="51"/>
+      <c r="T1" s="54"/>
+      <c r="U1" s="54"/>
       <c r="V1" s="19" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="W1" s="28" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="X1" s="4" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="Y1" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
     </row>
     <row r="2" spans="1:25">
@@ -4252,7 +4252,7 @@
         <v>10</v>
       </c>
       <c r="K2" s="10" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="L2" s="1" t="s">
         <v>107</v>
@@ -4261,16 +4261,16 @@
         <v>109</v>
       </c>
       <c r="N2" s="10" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="O2" s="1" t="s">
         <v>116</v>
       </c>
       <c r="X2" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="Y2" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
     </row>
     <row r="3" spans="1:25">
@@ -4308,7 +4308,7 @@
         <v>1</v>
       </c>
       <c r="L3" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="M3" t="s">
         <v>104</v>
@@ -4317,7 +4317,7 @@
         <v>1</v>
       </c>
       <c r="O3" s="23" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="S3">
         <v>1</v>
@@ -4329,16 +4329,16 @@
         <v>143</v>
       </c>
       <c r="V3" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="W3" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="X3" t="s">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="Y3" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
     </row>
     <row r="4" spans="1:25">
@@ -4376,7 +4376,7 @@
         <v>2</v>
       </c>
       <c r="L4" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="M4" t="s">
         <v>110</v>
@@ -4397,13 +4397,13 @@
         <v>145</v>
       </c>
       <c r="V4" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="W4" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="X4" t="s">
-        <v>399</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" spans="1:25">
@@ -4441,16 +4441,16 @@
         <v>3</v>
       </c>
       <c r="L5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="M5" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="N5">
         <v>3</v>
       </c>
       <c r="O5" s="23" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="S5">
         <v>3</v>
@@ -4462,13 +4462,13 @@
         <v>147</v>
       </c>
       <c r="V5" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="W5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="X5" t="s">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="6" spans="1:25">
@@ -4512,16 +4512,16 @@
         <v>4</v>
       </c>
       <c r="O6" s="23" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="V6" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="W6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="X6" t="s">
-        <v>401</v>
+        <v>400</v>
       </c>
     </row>
     <row r="7" spans="1:25">
@@ -4559,13 +4559,13 @@
         <v>121</v>
       </c>
       <c r="V7" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="W7" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="X7" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="1:25">
@@ -4585,7 +4585,7 @@
         <v>6</v>
       </c>
       <c r="I8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="J8" t="s">
         <v>31</v>
@@ -4594,7 +4594,7 @@
         <v>6</v>
       </c>
       <c r="L8" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="N8">
         <v>6</v>
@@ -4603,13 +4603,13 @@
         <v>122</v>
       </c>
       <c r="V8" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="W8" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="X8" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
     </row>
     <row r="9" spans="1:25">
@@ -4638,13 +4638,13 @@
         <v>118</v>
       </c>
       <c r="V9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="W9" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="X9" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
     </row>
     <row r="10" spans="1:25">
@@ -4667,13 +4667,13 @@
         <v>120</v>
       </c>
       <c r="V10" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="W10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="X10" t="s">
-        <v>405</v>
+        <v>404</v>
       </c>
     </row>
     <row r="11" spans="1:25">
@@ -4690,13 +4690,13 @@
         <v>12</v>
       </c>
       <c r="V11" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="W11" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="X11" t="s">
-        <v>406</v>
+        <v>405</v>
       </c>
     </row>
     <row r="12" spans="1:25">
@@ -4715,13 +4715,13 @@
       <c r="E12" s="10"/>
       <c r="F12" s="1"/>
       <c r="V12" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="W12" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="X12" t="s">
-        <v>407</v>
+        <v>406</v>
       </c>
     </row>
     <row r="13" spans="1:25">
@@ -4738,13 +4738,13 @@
         <v>12</v>
       </c>
       <c r="V13" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="W13" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="X13" t="s">
-        <v>408</v>
+        <v>407</v>
       </c>
     </row>
     <row r="14" spans="1:25">
@@ -4761,13 +4761,13 @@
         <v>12</v>
       </c>
       <c r="V14" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="W14" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="X14" t="s">
-        <v>409</v>
+        <v>408</v>
       </c>
     </row>
     <row r="15" spans="1:25">
@@ -4784,13 +4784,13 @@
         <v>12</v>
       </c>
       <c r="V15" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="W15" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="X15" t="s">
-        <v>410</v>
+        <v>409</v>
       </c>
     </row>
     <row r="16" spans="1:25">
@@ -4807,13 +4807,13 @@
         <v>12</v>
       </c>
       <c r="V16" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="W16" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="X16" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
     </row>
     <row r="17" spans="1:24">
@@ -4830,13 +4830,13 @@
         <v>12</v>
       </c>
       <c r="V17" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="W17" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="X17" t="s">
-        <v>412</v>
+        <v>411</v>
       </c>
     </row>
     <row r="18" spans="1:24">
@@ -4853,13 +4853,13 @@
         <v>12</v>
       </c>
       <c r="V18" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="W18" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="X18" t="s">
-        <v>413</v>
+        <v>412</v>
       </c>
     </row>
     <row r="19" spans="1:24">
@@ -4876,13 +4876,13 @@
         <v>12</v>
       </c>
       <c r="V19" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="W19" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="X19" t="s">
-        <v>414</v>
+        <v>413</v>
       </c>
     </row>
     <row r="20" spans="1:24">
@@ -4899,13 +4899,13 @@
         <v>12</v>
       </c>
       <c r="V20" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="W20" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="X20" t="s">
-        <v>415</v>
+        <v>414</v>
       </c>
     </row>
     <row r="21" spans="1:24">
@@ -4922,13 +4922,13 @@
         <v>12</v>
       </c>
       <c r="V21" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="W21" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="X21" t="s">
-        <v>416</v>
+        <v>415</v>
       </c>
     </row>
     <row r="22" spans="1:24">
@@ -4945,13 +4945,13 @@
         <v>12</v>
       </c>
       <c r="V22" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="W22" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="X22" t="s">
-        <v>417</v>
+        <v>416</v>
       </c>
     </row>
     <row r="23" spans="1:24">
@@ -4968,10 +4968,10 @@
         <v>12</v>
       </c>
       <c r="V23" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="X23" t="s">
-        <v>418</v>
+        <v>417</v>
       </c>
     </row>
     <row r="24" spans="1:24">
@@ -4988,13 +4988,13 @@
         <v>12</v>
       </c>
       <c r="V24" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="W24" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="X24" t="s">
-        <v>419</v>
+        <v>418</v>
       </c>
     </row>
     <row r="25" spans="1:24">
@@ -5011,13 +5011,13 @@
         <v>12</v>
       </c>
       <c r="V25" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="W25" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="X25" t="s">
-        <v>420</v>
+        <v>419</v>
       </c>
     </row>
     <row r="26" spans="1:24">
@@ -5034,13 +5034,13 @@
         <v>71</v>
       </c>
       <c r="V26" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="W26" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="X26" t="s">
-        <v>421</v>
+        <v>420</v>
       </c>
     </row>
     <row r="27" spans="1:24">
@@ -5057,13 +5057,13 @@
         <v>74</v>
       </c>
       <c r="V27" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="W27" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="X27" t="s">
-        <v>422</v>
+        <v>421</v>
       </c>
     </row>
     <row r="28" spans="1:24">
@@ -5080,13 +5080,13 @@
         <v>74</v>
       </c>
       <c r="V28" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="W28" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="X28" t="s">
-        <v>423</v>
+        <v>422</v>
       </c>
     </row>
     <row r="29" spans="1:24">
@@ -5103,13 +5103,13 @@
         <v>74</v>
       </c>
       <c r="V29" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="W29" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="X29" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
     </row>
     <row r="30" spans="1:24">
@@ -5126,13 +5126,13 @@
         <v>74</v>
       </c>
       <c r="V30" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="W30" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="X30" t="s">
-        <v>425</v>
+        <v>424</v>
       </c>
     </row>
     <row r="31" spans="1:24">
@@ -5146,13 +5146,13 @@
         <v>74</v>
       </c>
       <c r="V31" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="W31" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="X31" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="32" spans="1:24">
@@ -5166,13 +5166,13 @@
         <v>74</v>
       </c>
       <c r="V32" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="W32" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="X32" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="33" spans="1:24">
@@ -5189,10 +5189,10 @@
         <v>12</v>
       </c>
       <c r="W33" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="X33" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="34" spans="1:24">
@@ -5209,10 +5209,10 @@
         <v>12</v>
       </c>
       <c r="W34" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="X34" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="35" spans="1:24">
@@ -5229,10 +5229,10 @@
         <v>12</v>
       </c>
       <c r="W35" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="X35" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="36" spans="1:24">
@@ -5249,10 +5249,10 @@
         <v>12</v>
       </c>
       <c r="W36" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="X36" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="37" spans="1:24">
@@ -5269,10 +5269,10 @@
         <v>12</v>
       </c>
       <c r="W37" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="X37" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="38" spans="1:24">
@@ -5289,10 +5289,10 @@
         <v>12</v>
       </c>
       <c r="W38" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="X38" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="39" spans="1:24">
@@ -5309,10 +5309,10 @@
         <v>12</v>
       </c>
       <c r="W39" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="X39" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="40" spans="1:24">
@@ -5320,13 +5320,13 @@
         <v>47</v>
       </c>
       <c r="B40" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="W40" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="X40" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="41" spans="1:24">
@@ -5337,10 +5337,10 @@
         <v>70</v>
       </c>
       <c r="W41" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="X41" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="42" spans="1:24">
@@ -5348,13 +5348,13 @@
         <v>76</v>
       </c>
       <c r="B42" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="W42" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="X42" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="43" spans="1:24">
@@ -5362,10 +5362,10 @@
         <v>45</v>
       </c>
       <c r="B43" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="X43" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="44" spans="1:24">
@@ -5373,296 +5373,296 @@
         <v>72</v>
       </c>
       <c r="B44" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="W44" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="X44" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="45" spans="1:24">
       <c r="X45" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="46" spans="1:24">
       <c r="W46" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="X46" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="47" spans="1:24">
       <c r="W47" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="X47" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="48" spans="1:24">
       <c r="W48" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="X48" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="49" spans="1:24">
       <c r="W49" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="X49" t="s">
-        <v>444</v>
+        <v>443</v>
       </c>
     </row>
     <row r="50" spans="1:24">
       <c r="W50" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="X50" t="s">
-        <v>445</v>
+        <v>444</v>
       </c>
     </row>
     <row r="51" spans="1:24">
       <c r="W51" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="X51" t="s">
-        <v>446</v>
+        <v>445</v>
       </c>
     </row>
     <row r="52" spans="1:24">
       <c r="W52" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="X52" t="s">
-        <v>447</v>
+        <v>446</v>
       </c>
     </row>
     <row r="53" spans="1:24">
       <c r="W53" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="X53" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
     </row>
     <row r="54" spans="1:24">
       <c r="A54" s="1"/>
       <c r="W54" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="55" spans="1:24">
       <c r="W55" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="56" spans="1:24">
       <c r="W56" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="57" spans="1:24">
       <c r="W57" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="58" spans="1:24">
       <c r="W58" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="60" spans="1:24">
       <c r="W60" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
     </row>
     <row r="61" spans="1:24">
       <c r="W61" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
     </row>
     <row r="62" spans="1:24">
       <c r="W62" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="63" spans="1:24">
       <c r="W63" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
     </row>
     <row r="64" spans="1:24">
       <c r="W64" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
     </row>
     <row r="65" spans="23:23">
       <c r="W65" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
     </row>
     <row r="66" spans="23:23">
       <c r="W66" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="67" spans="23:23">
       <c r="W67" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="68" spans="23:23">
       <c r="W68" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
     </row>
     <row r="69" spans="23:23">
       <c r="W69" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="70" spans="23:23">
       <c r="W70" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
     </row>
     <row r="72" spans="23:23">
       <c r="W72" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
     </row>
     <row r="73" spans="23:23">
       <c r="W73" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
     </row>
     <row r="74" spans="23:23">
       <c r="W74" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="75" spans="23:23">
       <c r="W75" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
     </row>
     <row r="76" spans="23:23">
       <c r="W76" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
     </row>
     <row r="77" spans="23:23">
       <c r="W77" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
     </row>
     <row r="79" spans="23:23">
       <c r="W79" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
     </row>
     <row r="80" spans="23:23">
       <c r="W80" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
     </row>
     <row r="81" spans="23:23">
       <c r="W81" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
     <row r="82" spans="23:23">
       <c r="W82" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
     </row>
     <row r="83" spans="23:23">
       <c r="W83" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="84" spans="23:23">
       <c r="W84" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
     </row>
     <row r="85" spans="23:23">
       <c r="W85" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="86" spans="23:23">
       <c r="W86" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="87" spans="23:23">
       <c r="W87" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
     </row>
     <row r="88" spans="23:23">
       <c r="W88" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
     </row>
     <row r="90" spans="23:23">
       <c r="W90" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
     </row>
     <row r="91" spans="23:23">
       <c r="W91" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="93" spans="23:23">
       <c r="W93" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="94" spans="23:23">
       <c r="W94" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="95" spans="23:23">
       <c r="W95" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
     </row>
     <row r="96" spans="23:23">
       <c r="W96" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="105" spans="1:8">
       <c r="B105" t="s">
+        <v>198</v>
+      </c>
+      <c r="C105" t="s">
         <v>199</v>
       </c>
-      <c r="C105" t="s">
+      <c r="D105" t="s">
         <v>200</v>
       </c>
-      <c r="D105" t="s">
+      <c r="E105" t="s">
         <v>201</v>
       </c>
-      <c r="E105" t="s">
+      <c r="F105" t="s">
         <v>202</v>
       </c>
-      <c r="F105" t="s">
+      <c r="G105" t="s">
         <v>203</v>
       </c>
-      <c r="G105" t="s">
+      <c r="H105" t="s">
         <v>204</v>
-      </c>
-      <c r="H105" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="106" spans="1:8">
@@ -5670,13 +5670,13 @@
         <v>83</v>
       </c>
       <c r="B106" t="s">
+        <v>205</v>
+      </c>
+      <c r="C106" t="s">
         <v>206</v>
       </c>
-      <c r="C106" t="s">
+      <c r="D106" t="s">
         <v>207</v>
-      </c>
-      <c r="D106" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="107" spans="1:8">
@@ -5684,13 +5684,13 @@
         <v>86</v>
       </c>
       <c r="B107" t="s">
+        <v>208</v>
+      </c>
+      <c r="C107" t="s">
         <v>209</v>
       </c>
-      <c r="C107" t="s">
+      <c r="D107" t="s">
         <v>210</v>
-      </c>
-      <c r="D107" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="108" spans="1:8">
@@ -5698,13 +5698,13 @@
         <v>89</v>
       </c>
       <c r="B108" t="s">
+        <v>211</v>
+      </c>
+      <c r="C108" t="s">
         <v>212</v>
       </c>
-      <c r="C108" t="s">
+      <c r="D108" t="s">
         <v>213</v>
-      </c>
-      <c r="D108" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="109" spans="1:8">
@@ -5712,13 +5712,13 @@
         <v>92</v>
       </c>
       <c r="B109" t="s">
+        <v>214</v>
+      </c>
+      <c r="C109" t="s">
         <v>215</v>
       </c>
-      <c r="C109" t="s">
+      <c r="D109" t="s">
         <v>216</v>
-      </c>
-      <c r="D109" t="s">
-        <v>217</v>
       </c>
     </row>
     <row r="110" spans="1:8">
@@ -5726,13 +5726,13 @@
         <v>93</v>
       </c>
       <c r="B110" t="s">
+        <v>217</v>
+      </c>
+      <c r="C110" t="s">
         <v>218</v>
       </c>
-      <c r="C110" t="s">
+      <c r="D110" t="s">
         <v>219</v>
-      </c>
-      <c r="D110" t="s">
-        <v>220</v>
       </c>
     </row>
     <row r="111" spans="1:8">
@@ -5740,13 +5740,13 @@
         <v>94</v>
       </c>
       <c r="B111" t="s">
+        <v>220</v>
+      </c>
+      <c r="C111" t="s">
         <v>221</v>
       </c>
-      <c r="C111" t="s">
+      <c r="D111" t="s">
         <v>222</v>
-      </c>
-      <c r="D111" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="112" spans="1:8">
@@ -5754,13 +5754,13 @@
         <v>95</v>
       </c>
       <c r="B112" t="s">
+        <v>223</v>
+      </c>
+      <c r="C112" t="s">
         <v>224</v>
       </c>
-      <c r="C112" t="s">
+      <c r="D112" t="s">
         <v>225</v>
-      </c>
-      <c r="D112" t="s">
-        <v>226</v>
       </c>
     </row>
   </sheetData>

</xml_diff>